<commit_message>
chore: Update Purchase Request template file
- Modified the PurchaseRequestTemplate.xlsx to reflect the latest changes in the purchase request process, ensuring it meets current requirements and standards.
</commit_message>
<xml_diff>
--- a/storage/app/templates/PurchaseRequestTemplate.xlsx
+++ b/storage/app/templates/PurchaseRequestTemplate.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\CapstoneOJT\CagSU-SVP-System\storage\app\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\CapstoneCAGSUSVPSystem\storage\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32E3725B-A4FF-4D75-BB47-55712468AEBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8656DDA-1C46-4023-8A16-B3A972DE2E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -124,8 +124,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -579,8 +579,8 @@
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
@@ -619,10 +619,10 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -673,6 +673,129 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -691,136 +814,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1347,37 +1347,37 @@
       <c r="G2" s="31"/>
     </row>
     <row r="3" spans="1:7" ht="18">
-      <c r="A3" s="76" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="76"/>
-      <c r="C3" s="76"/>
-      <c r="D3" s="76"/>
-      <c r="E3" s="76"/>
-      <c r="F3" s="76"/>
-      <c r="G3" s="76"/>
+      <c r="A3" s="32" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
     </row>
     <row r="4" spans="1:7" ht="18.75" customHeight="1">
-      <c r="A4" s="77" t="s">
+      <c r="A4" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="77"/>
-      <c r="C4" s="77"/>
-      <c r="D4" s="77"/>
-      <c r="E4" s="77"/>
-      <c r="F4" s="77"/>
-      <c r="G4" s="77"/>
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="33"/>
     </row>
     <row r="5" spans="1:7" ht="15" customHeight="1">
-      <c r="A5" s="78" t="s">
+      <c r="A5" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="78"/>
-      <c r="C5" s="78"/>
-      <c r="D5" s="78"/>
-      <c r="E5" s="78"/>
-      <c r="F5" s="78"/>
-      <c r="G5" s="78"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
     </row>
     <row r="6" spans="1:7" ht="21" customHeight="1">
       <c r="A6" s="3" t="s">
@@ -1388,71 +1388,71 @@
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
-      <c r="E6" s="79" t="s">
+      <c r="E6" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="79"/>
-      <c r="G6" s="79"/>
+      <c r="F6" s="35"/>
+      <c r="G6" s="35"/>
     </row>
     <row r="7" spans="1:7" ht="18" customHeight="1">
-      <c r="A7" s="65"/>
-      <c r="B7" s="66"/>
+      <c r="A7" s="36"/>
+      <c r="B7" s="37"/>
       <c r="C7" s="5" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="7"/>
-      <c r="F7" s="67"/>
-      <c r="G7" s="68"/>
+      <c r="F7" s="38"/>
+      <c r="G7" s="39"/>
     </row>
     <row r="8" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A8" s="69" t="s">
+      <c r="A8" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="70"/>
-      <c r="C8" s="71" t="s">
+      <c r="B8" s="41"/>
+      <c r="C8" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="72"/>
-      <c r="E8" s="73"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="44"/>
       <c r="F8" s="8"/>
       <c r="G8" s="9"/>
     </row>
     <row r="9" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A9" s="40" t="s">
+      <c r="A9" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="75" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="40" t="s">
+      <c r="C9" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="41"/>
-      <c r="E9" s="34" t="s">
+      <c r="D9" s="80"/>
+      <c r="E9" s="75" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="34" t="s">
+      <c r="F9" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="34" t="s">
+      <c r="G9" s="75" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A10" s="42"/>
-      <c r="B10" s="35"/>
-      <c r="C10" s="42"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="35"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="35"/>
+      <c r="A10" s="48"/>
+      <c r="B10" s="76"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="81"/>
+      <c r="E10" s="76"/>
+      <c r="F10" s="76"/>
+      <c r="G10" s="76"/>
     </row>
     <row r="11" spans="1:7" ht="16.5" customHeight="1">
       <c r="A11" s="10"/>
       <c r="B11" s="11"/>
-      <c r="C11" s="74"/>
-      <c r="D11" s="75"/>
+      <c r="C11" s="45"/>
+      <c r="D11" s="46"/>
       <c r="E11" s="12"/>
       <c r="F11" s="13"/>
       <c r="G11" s="14">
@@ -1463,8 +1463,8 @@
     <row r="12" spans="1:7" ht="15" customHeight="1">
       <c r="A12" s="10"/>
       <c r="B12" s="11"/>
-      <c r="C12" s="63"/>
-      <c r="D12" s="64"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="50"/>
       <c r="E12" s="12"/>
       <c r="F12" s="13"/>
       <c r="G12" s="15">
@@ -1475,8 +1475,8 @@
     <row r="13" spans="1:7" ht="16.5" customHeight="1">
       <c r="A13" s="10"/>
       <c r="B13" s="11"/>
-      <c r="C13" s="63"/>
-      <c r="D13" s="64"/>
+      <c r="C13" s="49"/>
+      <c r="D13" s="50"/>
       <c r="E13" s="12"/>
       <c r="F13" s="13"/>
       <c r="G13" s="15">
@@ -1487,8 +1487,8 @@
     <row r="14" spans="1:7" ht="13.5" customHeight="1">
       <c r="A14" s="10"/>
       <c r="B14" s="11"/>
-      <c r="C14" s="63"/>
-      <c r="D14" s="64"/>
+      <c r="C14" s="49"/>
+      <c r="D14" s="50"/>
       <c r="E14" s="12"/>
       <c r="F14" s="13"/>
       <c r="G14" s="15">
@@ -1499,8 +1499,8 @@
     <row r="15" spans="1:7" ht="13.5" customHeight="1">
       <c r="A15" s="10"/>
       <c r="B15" s="11"/>
-      <c r="C15" s="63"/>
-      <c r="D15" s="64"/>
+      <c r="C15" s="49"/>
+      <c r="D15" s="50"/>
       <c r="E15" s="12"/>
       <c r="F15" s="13"/>
       <c r="G15" s="15">
@@ -1511,8 +1511,8 @@
     <row r="16" spans="1:7" ht="15" customHeight="1">
       <c r="A16" s="10"/>
       <c r="B16" s="11"/>
-      <c r="C16" s="63"/>
-      <c r="D16" s="64"/>
+      <c r="C16" s="49"/>
+      <c r="D16" s="50"/>
       <c r="E16" s="12"/>
       <c r="F16" s="13"/>
       <c r="G16" s="15">
@@ -1523,8 +1523,8 @@
     <row r="17" spans="1:7" ht="15" customHeight="1">
       <c r="A17" s="10"/>
       <c r="B17" s="11"/>
-      <c r="C17" s="63"/>
-      <c r="D17" s="64"/>
+      <c r="C17" s="49"/>
+      <c r="D17" s="50"/>
       <c r="E17" s="12"/>
       <c r="F17" s="13"/>
       <c r="G17" s="15">
@@ -1535,8 +1535,8 @@
     <row r="18" spans="1:7" ht="15" customHeight="1">
       <c r="A18" s="10"/>
       <c r="B18" s="11"/>
-      <c r="C18" s="63"/>
-      <c r="D18" s="64"/>
+      <c r="C18" s="49"/>
+      <c r="D18" s="50"/>
       <c r="E18" s="12"/>
       <c r="F18" s="13"/>
       <c r="G18" s="15">
@@ -1547,8 +1547,8 @@
     <row r="19" spans="1:7" ht="15" customHeight="1">
       <c r="A19" s="10"/>
       <c r="B19" s="11"/>
-      <c r="C19" s="63"/>
-      <c r="D19" s="64"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="50"/>
       <c r="E19" s="12"/>
       <c r="F19" s="13"/>
       <c r="G19" s="15">
@@ -1559,8 +1559,8 @@
     <row r="20" spans="1:7" ht="15" customHeight="1">
       <c r="A20" s="10"/>
       <c r="B20" s="11"/>
-      <c r="C20" s="63"/>
-      <c r="D20" s="64"/>
+      <c r="C20" s="49"/>
+      <c r="D20" s="50"/>
       <c r="E20" s="12"/>
       <c r="F20" s="13"/>
       <c r="G20" s="15">
@@ -1571,8 +1571,8 @@
     <row r="21" spans="1:7" ht="15" customHeight="1">
       <c r="A21" s="10"/>
       <c r="B21" s="11"/>
-      <c r="C21" s="63"/>
-      <c r="D21" s="64"/>
+      <c r="C21" s="49"/>
+      <c r="D21" s="50"/>
       <c r="E21" s="12"/>
       <c r="F21" s="13"/>
       <c r="G21" s="15">
@@ -1583,8 +1583,8 @@
     <row r="22" spans="1:7" ht="15" customHeight="1">
       <c r="A22" s="10"/>
       <c r="B22" s="11"/>
-      <c r="C22" s="63"/>
-      <c r="D22" s="64"/>
+      <c r="C22" s="49"/>
+      <c r="D22" s="50"/>
       <c r="E22" s="12"/>
       <c r="F22" s="13"/>
       <c r="G22" s="15">
@@ -1595,8 +1595,8 @@
     <row r="23" spans="1:7" ht="15" customHeight="1">
       <c r="A23" s="10"/>
       <c r="B23" s="11"/>
-      <c r="C23" s="63"/>
-      <c r="D23" s="64"/>
+      <c r="C23" s="49"/>
+      <c r="D23" s="50"/>
       <c r="E23" s="12"/>
       <c r="F23" s="13"/>
       <c r="G23" s="15">
@@ -1607,8 +1607,8 @@
     <row r="24" spans="1:7" ht="15" customHeight="1">
       <c r="A24" s="10"/>
       <c r="B24" s="11"/>
-      <c r="C24" s="63"/>
-      <c r="D24" s="64"/>
+      <c r="C24" s="49"/>
+      <c r="D24" s="50"/>
       <c r="E24" s="12"/>
       <c r="F24" s="13"/>
       <c r="G24" s="15">
@@ -1619,8 +1619,8 @@
     <row r="25" spans="1:7" ht="15" customHeight="1">
       <c r="A25" s="10"/>
       <c r="B25" s="11"/>
-      <c r="C25" s="63"/>
-      <c r="D25" s="64"/>
+      <c r="C25" s="49"/>
+      <c r="D25" s="50"/>
       <c r="E25" s="12"/>
       <c r="F25" s="13"/>
       <c r="G25" s="15">
@@ -1631,8 +1631,8 @@
     <row r="26" spans="1:7" ht="15" customHeight="1">
       <c r="A26" s="10"/>
       <c r="B26" s="11"/>
-      <c r="C26" s="63"/>
-      <c r="D26" s="64"/>
+      <c r="C26" s="49"/>
+      <c r="D26" s="50"/>
       <c r="E26" s="12"/>
       <c r="F26" s="13"/>
       <c r="G26" s="15">
@@ -1643,8 +1643,8 @@
     <row r="27" spans="1:7" ht="15" customHeight="1">
       <c r="A27" s="10"/>
       <c r="B27" s="11"/>
-      <c r="C27" s="63"/>
-      <c r="D27" s="64"/>
+      <c r="C27" s="49"/>
+      <c r="D27" s="50"/>
       <c r="E27" s="12"/>
       <c r="F27" s="13"/>
       <c r="G27" s="15">
@@ -1655,8 +1655,8 @@
     <row r="28" spans="1:7" ht="15" customHeight="1">
       <c r="A28" s="10"/>
       <c r="B28" s="11"/>
-      <c r="C28" s="63"/>
-      <c r="D28" s="64"/>
+      <c r="C28" s="49"/>
+      <c r="D28" s="50"/>
       <c r="E28" s="12"/>
       <c r="F28" s="13"/>
       <c r="G28" s="15">
@@ -1667,8 +1667,8 @@
     <row r="29" spans="1:7" ht="15" customHeight="1">
       <c r="A29" s="10"/>
       <c r="B29" s="11"/>
-      <c r="C29" s="44"/>
-      <c r="D29" s="45"/>
+      <c r="C29" s="51"/>
+      <c r="D29" s="52"/>
       <c r="E29" s="12"/>
       <c r="F29" s="13"/>
       <c r="G29" s="15">
@@ -1679,8 +1679,8 @@
     <row r="30" spans="1:7" ht="15" customHeight="1">
       <c r="A30" s="10"/>
       <c r="B30" s="11"/>
-      <c r="C30" s="44"/>
-      <c r="D30" s="45"/>
+      <c r="C30" s="51"/>
+      <c r="D30" s="52"/>
       <c r="E30" s="12"/>
       <c r="F30" s="13"/>
       <c r="G30" s="15">
@@ -1691,8 +1691,8 @@
     <row r="31" spans="1:7" ht="15" customHeight="1">
       <c r="A31" s="10"/>
       <c r="B31" s="11"/>
-      <c r="C31" s="44"/>
-      <c r="D31" s="45"/>
+      <c r="C31" s="51"/>
+      <c r="D31" s="52"/>
       <c r="E31" s="12"/>
       <c r="F31" s="13"/>
       <c r="G31" s="15">
@@ -1703,8 +1703,8 @@
     <row r="32" spans="1:7" ht="15" customHeight="1">
       <c r="A32" s="10"/>
       <c r="B32" s="11"/>
-      <c r="C32" s="44"/>
-      <c r="D32" s="45"/>
+      <c r="C32" s="51"/>
+      <c r="D32" s="52"/>
       <c r="E32" s="12"/>
       <c r="F32" s="13"/>
       <c r="G32" s="15">
@@ -1715,8 +1715,8 @@
     <row r="33" spans="1:7" ht="15" customHeight="1">
       <c r="A33" s="10"/>
       <c r="B33" s="11"/>
-      <c r="C33" s="44"/>
-      <c r="D33" s="45"/>
+      <c r="C33" s="51"/>
+      <c r="D33" s="52"/>
       <c r="E33" s="12"/>
       <c r="F33" s="13"/>
       <c r="G33" s="15">
@@ -1727,8 +1727,8 @@
     <row r="34" spans="1:7" ht="15" customHeight="1">
       <c r="A34" s="10"/>
       <c r="B34" s="11"/>
-      <c r="C34" s="44"/>
-      <c r="D34" s="45"/>
+      <c r="C34" s="51"/>
+      <c r="D34" s="52"/>
       <c r="E34" s="12"/>
       <c r="F34" s="13"/>
       <c r="G34" s="15">
@@ -1739,8 +1739,8 @@
     <row r="35" spans="1:7" ht="15" customHeight="1">
       <c r="A35" s="10"/>
       <c r="B35" s="11"/>
-      <c r="C35" s="44"/>
-      <c r="D35" s="45"/>
+      <c r="C35" s="51"/>
+      <c r="D35" s="52"/>
       <c r="E35" s="12"/>
       <c r="F35" s="13"/>
       <c r="G35" s="15">
@@ -1751,8 +1751,8 @@
     <row r="36" spans="1:7" ht="15" customHeight="1">
       <c r="A36" s="10"/>
       <c r="B36" s="11"/>
-      <c r="C36" s="44"/>
-      <c r="D36" s="45"/>
+      <c r="C36" s="51"/>
+      <c r="D36" s="52"/>
       <c r="E36" s="12"/>
       <c r="F36" s="13"/>
       <c r="G36" s="15">
@@ -1763,8 +1763,8 @@
     <row r="37" spans="1:7" ht="15" customHeight="1">
       <c r="A37" s="10"/>
       <c r="B37" s="11"/>
-      <c r="C37" s="44"/>
-      <c r="D37" s="45"/>
+      <c r="C37" s="51"/>
+      <c r="D37" s="52"/>
       <c r="E37" s="12"/>
       <c r="F37" s="13"/>
       <c r="G37" s="15">
@@ -1775,8 +1775,8 @@
     <row r="38" spans="1:7" ht="15" customHeight="1">
       <c r="A38" s="10"/>
       <c r="B38" s="11"/>
-      <c r="C38" s="44"/>
-      <c r="D38" s="45"/>
+      <c r="C38" s="51"/>
+      <c r="D38" s="52"/>
       <c r="E38" s="12"/>
       <c r="F38" s="13"/>
       <c r="G38" s="15">
@@ -1787,8 +1787,8 @@
     <row r="39" spans="1:7" ht="15" customHeight="1">
       <c r="A39" s="10"/>
       <c r="B39" s="11"/>
-      <c r="C39" s="44"/>
-      <c r="D39" s="45"/>
+      <c r="C39" s="51"/>
+      <c r="D39" s="52"/>
       <c r="E39" s="12"/>
       <c r="F39" s="13"/>
       <c r="G39" s="15">
@@ -1799,8 +1799,8 @@
     <row r="40" spans="1:7" ht="15" customHeight="1">
       <c r="A40" s="10"/>
       <c r="B40" s="11"/>
-      <c r="C40" s="44"/>
-      <c r="D40" s="45"/>
+      <c r="C40" s="51"/>
+      <c r="D40" s="52"/>
       <c r="E40" s="12"/>
       <c r="F40" s="13"/>
       <c r="G40" s="15">
@@ -1811,8 +1811,8 @@
     <row r="41" spans="1:7" ht="15" customHeight="1">
       <c r="A41" s="10"/>
       <c r="B41" s="11"/>
-      <c r="C41" s="44"/>
-      <c r="D41" s="45"/>
+      <c r="C41" s="51"/>
+      <c r="D41" s="52"/>
       <c r="E41" s="12"/>
       <c r="F41" s="13"/>
       <c r="G41" s="15">
@@ -1823,8 +1823,8 @@
     <row r="42" spans="1:7" ht="15" customHeight="1">
       <c r="A42" s="10"/>
       <c r="B42" s="11"/>
-      <c r="C42" s="44"/>
-      <c r="D42" s="45"/>
+      <c r="C42" s="51"/>
+      <c r="D42" s="52"/>
       <c r="E42" s="12"/>
       <c r="F42" s="13"/>
       <c r="G42" s="15">
@@ -1835,8 +1835,8 @@
     <row r="43" spans="1:7" ht="15" customHeight="1">
       <c r="A43" s="10"/>
       <c r="B43" s="11"/>
-      <c r="C43" s="44"/>
-      <c r="D43" s="45"/>
+      <c r="C43" s="51"/>
+      <c r="D43" s="52"/>
       <c r="E43" s="12"/>
       <c r="F43" s="13"/>
       <c r="G43" s="15">
@@ -1847,8 +1847,8 @@
     <row r="44" spans="1:7" ht="15" customHeight="1">
       <c r="A44" s="10"/>
       <c r="B44" s="11"/>
-      <c r="C44" s="44"/>
-      <c r="D44" s="45"/>
+      <c r="C44" s="51"/>
+      <c r="D44" s="52"/>
       <c r="E44" s="12"/>
       <c r="F44" s="13"/>
       <c r="G44" s="15">
@@ -1859,8 +1859,8 @@
     <row r="45" spans="1:7" ht="15" customHeight="1">
       <c r="A45" s="10"/>
       <c r="B45" s="11"/>
-      <c r="C45" s="44"/>
-      <c r="D45" s="45"/>
+      <c r="C45" s="51"/>
+      <c r="D45" s="52"/>
       <c r="E45" s="12"/>
       <c r="F45" s="13"/>
       <c r="G45" s="15">
@@ -1871,8 +1871,8 @@
     <row r="46" spans="1:7" ht="15" customHeight="1">
       <c r="A46" s="10"/>
       <c r="B46" s="11"/>
-      <c r="C46" s="44"/>
-      <c r="D46" s="45"/>
+      <c r="C46" s="51"/>
+      <c r="D46" s="52"/>
       <c r="E46" s="12"/>
       <c r="F46" s="13"/>
       <c r="G46" s="15">
@@ -1883,8 +1883,8 @@
     <row r="47" spans="1:7" ht="15" customHeight="1">
       <c r="A47" s="10"/>
       <c r="B47" s="11"/>
-      <c r="C47" s="44"/>
-      <c r="D47" s="45"/>
+      <c r="C47" s="51"/>
+      <c r="D47" s="52"/>
       <c r="E47" s="12"/>
       <c r="F47" s="13"/>
       <c r="G47" s="15">
@@ -1895,8 +1895,8 @@
     <row r="48" spans="1:7" ht="15" customHeight="1">
       <c r="A48" s="10"/>
       <c r="B48" s="11"/>
-      <c r="C48" s="44"/>
-      <c r="D48" s="45"/>
+      <c r="C48" s="51"/>
+      <c r="D48" s="52"/>
       <c r="E48" s="12"/>
       <c r="F48" s="13"/>
       <c r="G48" s="15">
@@ -1907,8 +1907,8 @@
     <row r="49" spans="1:7" ht="15" customHeight="1">
       <c r="A49" s="10"/>
       <c r="B49" s="11"/>
-      <c r="C49" s="44"/>
-      <c r="D49" s="45"/>
+      <c r="C49" s="51"/>
+      <c r="D49" s="52"/>
       <c r="E49" s="12"/>
       <c r="F49" s="13"/>
       <c r="G49" s="15">
@@ -1919,8 +1919,8 @@
     <row r="50" spans="1:7" ht="15" customHeight="1">
       <c r="A50" s="10"/>
       <c r="B50" s="11"/>
-      <c r="C50" s="44"/>
-      <c r="D50" s="45"/>
+      <c r="C50" s="51"/>
+      <c r="D50" s="52"/>
       <c r="E50" s="12"/>
       <c r="F50" s="13"/>
       <c r="G50" s="15">
@@ -1931,8 +1931,8 @@
     <row r="51" spans="1:7" ht="15" customHeight="1">
       <c r="A51" s="10"/>
       <c r="B51" s="11"/>
-      <c r="C51" s="44"/>
-      <c r="D51" s="45"/>
+      <c r="C51" s="51"/>
+      <c r="D51" s="52"/>
       <c r="E51" s="12"/>
       <c r="F51" s="13"/>
       <c r="G51" s="15">
@@ -1943,8 +1943,8 @@
     <row r="52" spans="1:7" ht="15" customHeight="1">
       <c r="A52" s="10"/>
       <c r="B52" s="11"/>
-      <c r="C52" s="44"/>
-      <c r="D52" s="45"/>
+      <c r="C52" s="51"/>
+      <c r="D52" s="52"/>
       <c r="E52" s="12"/>
       <c r="F52" s="13"/>
       <c r="G52" s="15">
@@ -1955,8 +1955,8 @@
     <row r="53" spans="1:7" ht="15" customHeight="1">
       <c r="A53" s="10"/>
       <c r="B53" s="11"/>
-      <c r="C53" s="44"/>
-      <c r="D53" s="45"/>
+      <c r="C53" s="51"/>
+      <c r="D53" s="52"/>
       <c r="E53" s="12"/>
       <c r="F53" s="13"/>
       <c r="G53" s="15">
@@ -1967,8 +1967,8 @@
     <row r="54" spans="1:7" ht="15" customHeight="1">
       <c r="A54" s="10"/>
       <c r="B54" s="11"/>
-      <c r="C54" s="44"/>
-      <c r="D54" s="45"/>
+      <c r="C54" s="51"/>
+      <c r="D54" s="52"/>
       <c r="E54" s="12"/>
       <c r="F54" s="13"/>
       <c r="G54" s="15">
@@ -1979,8 +1979,8 @@
     <row r="55" spans="1:7" ht="15" customHeight="1">
       <c r="A55" s="10"/>
       <c r="B55" s="11"/>
-      <c r="C55" s="61"/>
-      <c r="D55" s="62"/>
+      <c r="C55" s="69"/>
+      <c r="D55" s="70"/>
       <c r="E55" s="12"/>
       <c r="F55" s="13"/>
       <c r="G55" s="15">
@@ -1991,8 +1991,8 @@
     <row r="56" spans="1:7">
       <c r="A56" s="10"/>
       <c r="B56" s="11"/>
-      <c r="C56" s="80"/>
-      <c r="D56" s="81"/>
+      <c r="C56" s="71"/>
+      <c r="D56" s="72"/>
       <c r="E56" s="12"/>
       <c r="F56" s="13"/>
       <c r="G56" s="15"/>
@@ -2000,10 +2000,10 @@
     <row r="57" spans="1:7" ht="15" customHeight="1">
       <c r="A57" s="16"/>
       <c r="B57" s="16"/>
-      <c r="C57" s="54" t="s">
+      <c r="C57" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="D57" s="55"/>
+      <c r="D57" s="57"/>
       <c r="E57" s="17"/>
       <c r="F57" s="18"/>
       <c r="G57" s="15">
@@ -2012,57 +2012,57 @@
       </c>
     </row>
     <row r="58" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A58" s="32" t="s">
+      <c r="A58" s="73" t="s">
         <v>16</v>
       </c>
-      <c r="B58" s="36" t="s">
+      <c r="B58" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="C58" s="36"/>
-      <c r="D58" s="36"/>
-      <c r="E58" s="36"/>
-      <c r="F58" s="36"/>
-      <c r="G58" s="37"/>
+      <c r="C58" s="77"/>
+      <c r="D58" s="77"/>
+      <c r="E58" s="77"/>
+      <c r="F58" s="77"/>
+      <c r="G58" s="78"/>
     </row>
     <row r="59" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A59" s="33"/>
-      <c r="B59" s="38"/>
-      <c r="C59" s="38"/>
-      <c r="D59" s="38"/>
-      <c r="E59" s="38"/>
-      <c r="F59" s="38"/>
-      <c r="G59" s="39"/>
+      <c r="A59" s="74"/>
+      <c r="B59" s="61"/>
+      <c r="C59" s="61"/>
+      <c r="D59" s="61"/>
+      <c r="E59" s="61"/>
+      <c r="F59" s="61"/>
+      <c r="G59" s="79"/>
     </row>
     <row r="60" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A60" s="33"/>
-      <c r="B60" s="38"/>
-      <c r="C60" s="38"/>
-      <c r="D60" s="38"/>
-      <c r="E60" s="38"/>
-      <c r="F60" s="38"/>
-      <c r="G60" s="39"/>
+      <c r="A60" s="74"/>
+      <c r="B60" s="61"/>
+      <c r="C60" s="61"/>
+      <c r="D60" s="61"/>
+      <c r="E60" s="61"/>
+      <c r="F60" s="61"/>
+      <c r="G60" s="79"/>
     </row>
     <row r="61" spans="1:7" hidden="1">
-      <c r="A61" s="33"/>
-      <c r="B61" s="38"/>
-      <c r="C61" s="38"/>
-      <c r="D61" s="38"/>
-      <c r="E61" s="38"/>
-      <c r="F61" s="38"/>
-      <c r="G61" s="39"/>
+      <c r="A61" s="74"/>
+      <c r="B61" s="61"/>
+      <c r="C61" s="61"/>
+      <c r="D61" s="61"/>
+      <c r="E61" s="61"/>
+      <c r="F61" s="61"/>
+      <c r="G61" s="79"/>
     </row>
     <row r="62" spans="1:7" ht="18" customHeight="1">
       <c r="A62" s="20"/>
-      <c r="B62" s="56" t="s">
+      <c r="B62" s="58" t="s">
         <v>18</v>
       </c>
-      <c r="C62" s="56"/>
+      <c r="C62" s="58"/>
       <c r="D62" s="21"/>
-      <c r="E62" s="57" t="s">
+      <c r="E62" s="59" t="s">
         <v>19</v>
       </c>
-      <c r="F62" s="57"/>
-      <c r="G62" s="58"/>
+      <c r="F62" s="59"/>
+      <c r="G62" s="60"/>
     </row>
     <row r="63" spans="1:7" ht="16.5" customHeight="1">
       <c r="A63" s="22"/>
@@ -2086,51 +2086,51 @@
       <c r="A65" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="B65" s="38"/>
-      <c r="C65" s="38"/>
+      <c r="B65" s="61"/>
+      <c r="C65" s="61"/>
       <c r="D65" s="19"/>
-      <c r="E65" s="59"/>
-      <c r="F65" s="59"/>
-      <c r="G65" s="60"/>
+      <c r="E65" s="62"/>
+      <c r="F65" s="62"/>
+      <c r="G65" s="63"/>
     </row>
     <row r="66" spans="1:7" ht="26.25" customHeight="1">
       <c r="A66" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="B66" s="46" t="s">
+      <c r="B66" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="46"/>
+      <c r="C66" s="64"/>
       <c r="D66" s="19"/>
-      <c r="E66" s="46" t="s">
+      <c r="E66" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="F66" s="46"/>
-      <c r="G66" s="47"/>
+      <c r="F66" s="64"/>
+      <c r="G66" s="65"/>
     </row>
     <row r="67" spans="1:7" ht="26.25" customHeight="1">
       <c r="A67" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="B67" s="48" t="s">
+      <c r="B67" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="C67" s="48"/>
+      <c r="C67" s="66"/>
       <c r="D67" s="26"/>
-      <c r="E67" s="49" t="s">
+      <c r="E67" s="67" t="s">
         <v>26</v>
       </c>
-      <c r="F67" s="49"/>
-      <c r="G67" s="50"/>
+      <c r="F67" s="67"/>
+      <c r="G67" s="68"/>
     </row>
     <row r="68" spans="1:7" ht="20.25" customHeight="1">
-      <c r="A68" s="51"/>
-      <c r="B68" s="52"/>
-      <c r="C68" s="52"/>
-      <c r="D68" s="52"/>
-      <c r="E68" s="52"/>
-      <c r="F68" s="52"/>
-      <c r="G68" s="53"/>
+      <c r="A68" s="53"/>
+      <c r="B68" s="54"/>
+      <c r="C68" s="54"/>
+      <c r="D68" s="54"/>
+      <c r="E68" s="54"/>
+      <c r="F68" s="54"/>
+      <c r="G68" s="55"/>
     </row>
     <row r="69" spans="1:7" ht="20.25" customHeight="1">
       <c r="A69" s="27"/>
@@ -2143,64 +2143,6 @@
     </row>
   </sheetData>
   <mergeCells count="74">
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="A68:G68"/>
-    <mergeCell ref="C57:D57"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="E62:G62"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="E65:G65"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="E66:G66"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="E67:G67"/>
-    <mergeCell ref="C52:D52"/>
-    <mergeCell ref="C53:D53"/>
-    <mergeCell ref="C54:D54"/>
-    <mergeCell ref="C55:D55"/>
-    <mergeCell ref="C56:D56"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="C48:D48"/>
-    <mergeCell ref="C49:D49"/>
-    <mergeCell ref="C50:D50"/>
-    <mergeCell ref="C51:D51"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="A58:A61"/>
     <mergeCell ref="B9:B10"/>
@@ -2217,13 +2159,68 @@
     <mergeCell ref="C31:D31"/>
     <mergeCell ref="C32:D32"/>
     <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="C48:D48"/>
+    <mergeCell ref="C49:D49"/>
+    <mergeCell ref="C50:D50"/>
+    <mergeCell ref="C51:D51"/>
+    <mergeCell ref="C52:D52"/>
+    <mergeCell ref="C53:D53"/>
+    <mergeCell ref="C54:D54"/>
+    <mergeCell ref="C55:D55"/>
+    <mergeCell ref="C56:D56"/>
+    <mergeCell ref="A68:G68"/>
+    <mergeCell ref="C57:D57"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="E62:G62"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="E65:G65"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="E66:G66"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="E67:G67"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:E8"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="E6:G6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.39370078740157483" right="0.27559055118110237" top="0.59055118110236227" bottom="0.51181102362204722" header="0" footer="0.51181102362204722"/>
+  <pageMargins left="0.39370078740157499" right="0.27559055118110198" top="0.59055118110236204" bottom="0.511811023622047" header="0" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="70" fitToHeight="10" orientation="portrait" r:id="rId1"/>
-  <headerFooter>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12 151</oddFooter>
-  </headerFooter>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="8" min="1" max="69" man="1"/>
   </colBreaks>

</xml_diff>